<commit_message>
demo: add oncho form
</commit_message>
<xml_diff>
--- a/Demo/LF/lf/demo_lf_tas_9999_2_part.xlsx
+++ b/Demo/LF/lf/demo_lf_tas_9999_2_part.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\lf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\LF\lf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E2E1098-C527-49BE-B519-5A0BC402F3E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47F6FCC-3DA9-4450-8C5E-141656769460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,20 @@
     <sheet name="choices" sheetId="2" r:id="rId2"/>
     <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>